<commit_message>
Document ECS deployment and repo guidance
Add CLAUDE.md with the repository architecture, commands, and operational guidance for working in this codebase. Update README to reflect the current admin-role checks, CI/CD flow, ECS deployment model, and expanded test coverage. Refresh the committed Excel fixture used by the upload normaliser tests.
</commit_message>
<xml_diff>
--- a/uploads/IS1.xlsx
+++ b/uploads/IS1.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1" showInkAnnotation="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1215BB3D-5FB5-4D73-8839-4DCF8CD492AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E666A45C-421C-420A-ABF5-464B36E1BAD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="750" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Income statement" sheetId="2" r:id="rId1"/>
@@ -1028,7 +1028,7 @@
       <c r="D3" s="12"/>
       <c r="E3" s="21"/>
       <c r="F3" s="41">
-        <v>45882</v>
+        <v>46278</v>
       </c>
       <c r="G3" s="3"/>
       <c r="H3" s="44"/>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="25">
-        <v>10000</v>
+        <v>1000</v>
       </c>
       <c r="F7" s="32"/>
       <c r="G7" s="3"/>
@@ -1095,7 +1095,7 @@
       <c r="E8" s="20"/>
       <c r="F8" s="32">
         <f>IF(OR(E6&lt;&gt;0,E7&lt;&gt;0),SUM(E6-E7),0)</f>
-        <v>590000</v>
+        <v>599000</v>
       </c>
       <c r="G8" s="3"/>
       <c r="H8" s="44"/>
@@ -1256,7 +1256,7 @@
       <c r="E20" s="20"/>
       <c r="F20" s="32">
         <f>IF(OR(Net_Sales,COGS),Net_Sales-COGS,0)</f>
-        <v>517000</v>
+        <v>526000</v>
       </c>
       <c r="G20" s="3"/>
       <c r="H20" s="44"/>
@@ -1682,7 +1682,7 @@
       <c r="E51" s="20"/>
       <c r="F51" s="35">
         <f>IF(OR(Gross_Profit,Total_Expenses),Gross_Profit-Total_Expenses,0)</f>
-        <v>360700</v>
+        <v>369700</v>
       </c>
       <c r="G51" s="3"/>
       <c r="H51" s="44"/>
@@ -1772,7 +1772,7 @@
       <c r="E58" s="20"/>
       <c r="F58" s="35">
         <f>IF(OR(Op_Income,Other_Income),Op_Income+Other_Income,0)</f>
-        <v>420700</v>
+        <v>429700</v>
       </c>
       <c r="G58" s="3"/>
       <c r="H58" s="44"/>
@@ -1901,6 +1901,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="26" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ac37c1753acd5e330d2062ccec26ea66">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3b340c7101c92c5120abd06486f94548" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -2200,15 +2209,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B25903B0-7748-4EC8-9AE6-30C7129DC7C9}">
   <ds:schemaRefs>
@@ -2229,6 +2229,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{078BDA64-E289-47E3-BE11-83ECE4B2E315}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{40E5EBD5-9A8B-4FB3-9210-57091BDE8FDC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2249,14 +2257,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{078BDA64-E289-47E3-BE11-83ECE4B2E315}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata"/>
 </file>
</xml_diff>

<commit_message>
Restore the IS1.xlsx test fixture
a36e7f7 committed an edited copy of the Excel test fixture (report date
moved to Sep-26 and figures changed so line items no longer reconcile to
the total), which failed four Excel normaliser tests and stopped the
deploy at the test step. Restores the workbook from 20e8bfd.
</commit_message>
<xml_diff>
--- a/uploads/IS1.xlsx
+++ b/uploads/IS1.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" showInkAnnotation="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E666A45C-421C-420A-ABF5-464B36E1BAD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1215BB3D-5FB5-4D73-8839-4DCF8CD492AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="750" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Income statement" sheetId="2" r:id="rId1"/>
@@ -1028,7 +1028,7 @@
       <c r="D3" s="12"/>
       <c r="E3" s="21"/>
       <c r="F3" s="41">
-        <v>46278</v>
+        <v>45882</v>
       </c>
       <c r="G3" s="3"/>
       <c r="H3" s="44"/>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="25">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="F7" s="32"/>
       <c r="G7" s="3"/>
@@ -1095,7 +1095,7 @@
       <c r="E8" s="20"/>
       <c r="F8" s="32">
         <f>IF(OR(E6&lt;&gt;0,E7&lt;&gt;0),SUM(E6-E7),0)</f>
-        <v>599000</v>
+        <v>590000</v>
       </c>
       <c r="G8" s="3"/>
       <c r="H8" s="44"/>
@@ -1256,7 +1256,7 @@
       <c r="E20" s="20"/>
       <c r="F20" s="32">
         <f>IF(OR(Net_Sales,COGS),Net_Sales-COGS,0)</f>
-        <v>526000</v>
+        <v>517000</v>
       </c>
       <c r="G20" s="3"/>
       <c r="H20" s="44"/>
@@ -1682,7 +1682,7 @@
       <c r="E51" s="20"/>
       <c r="F51" s="35">
         <f>IF(OR(Gross_Profit,Total_Expenses),Gross_Profit-Total_Expenses,0)</f>
-        <v>369700</v>
+        <v>360700</v>
       </c>
       <c r="G51" s="3"/>
       <c r="H51" s="44"/>
@@ -1772,7 +1772,7 @@
       <c r="E58" s="20"/>
       <c r="F58" s="35">
         <f>IF(OR(Op_Income,Other_Income),Op_Income+Other_Income,0)</f>
-        <v>429700</v>
+        <v>420700</v>
       </c>
       <c r="G58" s="3"/>
       <c r="H58" s="44"/>
@@ -1901,15 +1901,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="26" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ac37c1753acd5e330d2062ccec26ea66">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3b340c7101c92c5120abd06486f94548" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -2209,6 +2200,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B25903B0-7748-4EC8-9AE6-30C7129DC7C9}">
   <ds:schemaRefs>
@@ -2229,14 +2229,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{078BDA64-E289-47E3-BE11-83ECE4B2E315}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{40E5EBD5-9A8B-4FB3-9210-57091BDE8FDC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2257,6 +2249,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{078BDA64-E289-47E3-BE11-83ECE4B2E315}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata"/>
 </file>
</xml_diff>